<commit_message>
NRI-0009: rework xlsx import into one five-sheet workbook with cross-sheet links, pre-analysis, name upsert, transactional apply and template download, sync specs and archive change
</commit_message>
<xml_diff>
--- a/tests/fixtures/import_sample.xlsx
+++ b/tests/fixtures/import_sample.xlsx
@@ -7,7 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="события" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="События" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Персонажи" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Локации" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Организации" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Предметы" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,7 +20,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -46,8 +52,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,33 +420,63 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>Имя</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>start_date</t>
+          <t>Дата начала</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>end_date</t>
+          <t>Дата конца</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>characteristics</t>
+          <t>Характеристики</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>backstory</t>
+          <t>Предыстория</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Рейтинг</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Тип</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Связь персонажами</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Связь организациями</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Связь предметами</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Связь локациями</t>
         </is>
       </c>
     </row>
@@ -449,14 +486,12 @@
           <t>Взятие Штурмграда</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>1200-05-01</t>
-        </is>
+      <c r="B2" s="1" t="n">
+        <v>-255547</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>1200-05-14</t>
+          <t>1200-09-15</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -467,6 +502,31 @@
       <c r="E2" t="inlineStr">
         <is>
           <t>Город пал после разрушения стены</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Война</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Иван Ковач; Марта</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Гильдия копья</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Штурмовой щит; Амулет вдовы</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Штурмград</t>
         </is>
       </c>
     </row>
@@ -478,12 +538,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1200-06-15</t>
+          <t>1202-06-10</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>1200-07-01</t>
+          <t>1203-01-20</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -491,7 +551,619 @@
           <t>Тридцать верблюдов и охрана</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Поход</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Иван Ковач</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Карта востока; Амулет вдовы</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Восточный тракт</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Пир в ратуше</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>31.12.2025</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Имя</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Дата начала</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Дата конца</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Характеристики</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Предыстория</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Рейтинг</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>personality</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>tasks</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>music_url</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Изображение</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Связь событиями</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Связь организациями</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Связь предметами</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Связь локациями</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Иван Ковач</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="n">
+        <v>-262913</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Городской кузнец</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>4</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Упрямый</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Сковать парадные доспехи</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Взятие Штурмграда; Поход каравана на восток</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Карта востока</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Штурмград</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Марта</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>1185-07-20</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Предприимчивая торговка</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Взятие Штурмграда</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Штурмград</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Старый Кузнец</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>1160-01-01</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Молчалив, знает все ходы</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>3</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Взятие Штурмграда</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Старый Кузнец</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>1161-02-02</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Бывший капитан городской стражи</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Поход каравана на восток</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Гоблин-наёмник</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>1201-01-01</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Имя</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Дата начала</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Дата конца</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Характеристики</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Предыстория</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Рейтинг</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>tasks</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>music_url</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Изображение</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Связь событиями</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Связь персонажами</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Связь организациями</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Связь предметами</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Штурмград</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1100-01-01</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Обнесённая стеной крепость</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Взятие Штурмграда</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Иван Ковач; Марта</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Восточный тракт</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>1100-01-01</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Пыльный путь к восточным рынкам</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Поход каравана на восток</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Имя</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Дата начала</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Дата конца</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Характеристики</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Предыстория</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Рейтинг</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>tasks</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>music_url</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Изображение</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Связь событиями</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Связь персонажами</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Связь предметами</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Связь локациями</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Гильдия копья</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1150-01-01</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Наёмники и ремесленники старого города</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Взятие Штурмграда</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Иван Ковач</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Имя</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Дата начала</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Дата конца</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Характеристики</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Предыстория</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Рейтинг</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>music_url</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Связь событиями</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Связь персонажами</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Связь организациями</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Связь локациями</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Штурмовой щит</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1195-01-01</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Калёный щит с клёпаным краем</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Взятие Штурмграда</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Иван Ковач</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Карта востока</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>1201-01-01</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Выцветшая купеческая карта</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Поход каравана на восток</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Иван Ковач</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
NRI-0027: teach the xlsx import subevents and time — optional «Время начала» and «Родительское событие» columns on the События sheet with calendar-bound time parsing (warning, never a lost row), ghost-free two-level parent resolution through the shared domain judge in event_nesting.py, template examples and dialog hint covering both columns, the unreachable output_budget double-check removed as PR-035 gate debt, full isolated gate green 275/275 at 100% coverage, xlsx-import spec synced and the change archived
</commit_message>
<xml_diff>
--- a/tests/fixtures/import_sample.xlsx
+++ b/tests/fixtures/import_sample.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,45 +436,55 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>Время начала</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>Дата конца</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Характеристики</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Предыстория</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Рейтинг</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Тип</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Родительское событие</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
         <is>
           <t>Связь персонажами</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Связь организациями</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Связь предметами</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Связь локациями</t>
         </is>
@@ -489,42 +499,42 @@
       <c r="B2" s="1" t="n">
         <v>-255547</v>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>1200-09-15</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Осада длилась три недели</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Город пал после разрушения стены</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Война</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Иван Ковач; Марта</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Гильдия копья</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>Штурмовой щит; Амулет вдовы</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>Штурмград</t>
         </is>
@@ -541,32 +551,32 @@
           <t>1202-06-10</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>1203-01-20</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Тридцать верблюдов и охрана</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>Поход</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>Иван Ковач</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>Карта востока; Амулет вдовы</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>Восточный тракт</t>
         </is>

</xml_diff>